<commit_message>
Mark Adrian's dinner share settled
His 1,254 JPY comes out of receivables: the expense row flips from a
receivable to a repaid pill, the settlement card to a tick, and the
status band drops from 27,886.88 PHP owed to 27,404.09 across Eugene,
Kim and VM.

The workbook's Owed to Russel tab keeps Adrian's block for the record
but excludes it from the total, which is relabelled Total Still Owed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0153ymvRJsG2ELDmVi2KTRKy
</commit_message>
<xml_diff>
--- a/artifacts/japan-2026-07/Russel-inventory-2026-07.xlsx
+++ b/artifacts/japan-2026-07/Russel-inventory-2026-07.xlsx
@@ -9176,7 +9176,7 @@
     <row r="40">
       <c r="A40" s="22" t="inlineStr">
         <is>
-          <t>ADRIAN — 1 item</t>
+          <t>ADRIAN — SETTLED</t>
         </is>
       </c>
     </row>
@@ -9220,7 +9220,7 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>びっくりドンキー 道頓堀</t>
+          <t>びっくりドンキー 道頓堀 — PAID</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
@@ -9260,25 +9260,25 @@
     <row r="44">
       <c r="A44" s="21" t="inlineStr">
         <is>
-          <t>Not requested on this tab, included because it is outstanding on the same basis.</t>
+          <t>Settled. Shown for the record; excluded from the total below.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="17" t="inlineStr">
         <is>
-          <t>TOTAL OWED TO RUSSEL</t>
+          <t>TOTAL STILL OWED</t>
         </is>
       </c>
       <c r="B46" s="18" t="n"/>
       <c r="C46" s="18" t="n"/>
       <c r="D46" s="19">
-        <f>D19+D26+D37+D43</f>
+        <f>D19+D26+D37</f>
         <v/>
       </c>
       <c r="E46" s="18" t="n"/>
       <c r="F46" s="20">
-        <f>F19+F26+F37+F43</f>
+        <f>F19+F26+F37</f>
         <v/>
       </c>
     </row>

</xml_diff>